<commit_message>
Added testcase of generator portal login
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/abae56211fdd6e11/Desktop/Octopus saas/Excwl sheet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="13_ncr:801_{2AC28ABD-5620-4052-9C7E-703FCFC9F1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11BF205E-A572-4E86-936F-9558795B1EBB}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="13_ncr:801_{2AC28ABD-5620-4052-9C7E-703FCFC9F1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDB39C4F-F7CB-409C-88A3-D9B3D3D06BA3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="SatelliteLocation" sheetId="8" r:id="rId10"/>
     <sheet name="LiveView" sheetId="9" r:id="rId11"/>
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId12"/>
+    <sheet name="GeneratorPortal" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1337" uniqueCount="843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1359" uniqueCount="855">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -2578,6 +2579,42 @@
   </si>
   <si>
     <t>Email with valid format</t>
+  </si>
+  <si>
+    <t>Email with Alphabets</t>
+  </si>
+  <si>
+    <t>Email with Numbers</t>
+  </si>
+  <si>
+    <t>Email with Specialcharacters</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>765677</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Password with Alphabets </t>
+  </si>
+  <si>
+    <t>Password with Numbers</t>
+  </si>
+  <si>
+    <t>henrry123@gmail.com</t>
+  </si>
+  <si>
+    <t>henrry123#@gmail,com</t>
+  </si>
+  <si>
+    <t>Password with Specialcharacters</t>
+  </si>
+  <si>
+    <t>Password with all Characters</t>
+  </si>
+  <si>
+    <t>Henry123!@</t>
   </si>
 </sst>
 </file>
@@ -5098,6 +5135,101 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0512D46C-65A2-499B-8C92-EB4BEF7A1CC2}">
+  <dimension ref="CY1:DD5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="104" max="104" width="24.85546875" customWidth="1"/>
+    <col min="105" max="105" width="23.42578125" customWidth="1"/>
+    <col min="106" max="106" width="34.7109375" customWidth="1"/>
+    <col min="107" max="107" width="29.28515625" customWidth="1"/>
+    <col min="108" max="108" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="103:108" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="CY1" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="CZ1" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="DA1" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="DB1" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="DC1" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="DD1" s="3" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="2" spans="103:108" x14ac:dyDescent="0.25">
+      <c r="CY2" t="s">
+        <v>846</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>320</v>
+      </c>
+      <c r="DA2" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>238</v>
+      </c>
+      <c r="DC2" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="DD2" s="2" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="4" spans="103:108" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="CY4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="CZ4" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="DA4" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="DB4" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="DC4" s="3" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="5" spans="103:108" x14ac:dyDescent="0.25">
+      <c r="CY5" t="s">
+        <v>743</v>
+      </c>
+      <c r="CZ5" t="s">
+        <v>320</v>
+      </c>
+      <c r="DA5" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="DB5" t="s">
+        <v>238</v>
+      </c>
+      <c r="DC5" t="s">
+        <v>854</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="DD2" r:id="rId1" xr:uid="{94B42F2C-7046-4CDC-A622-B6682B8F51EB}"/>
+    <hyperlink ref="DC2" r:id="rId2" xr:uid="{F2801E8D-6087-460A-A710-A7B5F06DC167}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77142416-745D-4F9D-B8CB-E786E8AF6BF4}">
   <dimension ref="A1:D3"/>

</xml_diff>

<commit_message>
Added new class on generator portal login package
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -3,31 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="13_ncr:801_{2AC28ABD-5620-4052-9C7E-703FCFC9F1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDB39C4F-F7CB-409C-88A3-D9B3D3D06BA3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{0BC689DE-60D1-4641-9AF1-C6A0A8F0DCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Signup365" sheetId="1" r:id="rId1"/>
-    <sheet name="Generator" sheetId="10" r:id="rId2"/>
-    <sheet name="Routeassignment" sheetId="3" r:id="rId3"/>
-    <sheet name="Disposal Facillity" sheetId="11" r:id="rId4"/>
-    <sheet name="Unapplied checks" sheetId="12" r:id="rId5"/>
-    <sheet name="TransporterProfile" sheetId="2" r:id="rId6"/>
-    <sheet name="MyProfile" sheetId="4" r:id="rId7"/>
-    <sheet name="Drivers" sheetId="5" r:id="rId8"/>
-    <sheet name="Servicevehicle" sheetId="6" r:id="rId9"/>
-    <sheet name="SatelliteLocation" sheetId="8" r:id="rId10"/>
-    <sheet name="LiveView" sheetId="9" r:id="rId11"/>
-    <sheet name="GeneratorInformation" sheetId="7" r:id="rId12"/>
-    <sheet name="GeneratorPortal" sheetId="13" r:id="rId13"/>
+    <sheet name="GeneratorPortal" sheetId="14" r:id="rId1"/>
+    <sheet name="Signup365" sheetId="1" r:id="rId2"/>
+    <sheet name="Generator" sheetId="10" r:id="rId3"/>
+    <sheet name="Routeassignment" sheetId="3" r:id="rId4"/>
+    <sheet name="Disposal Facillity" sheetId="11" r:id="rId5"/>
+    <sheet name="Unapplied checks" sheetId="12" r:id="rId6"/>
+    <sheet name="TransporterProfile" sheetId="2" r:id="rId7"/>
+    <sheet name="MyProfile" sheetId="4" r:id="rId8"/>
+    <sheet name="Drivers" sheetId="5" r:id="rId9"/>
+    <sheet name="Servicevehicle" sheetId="6" r:id="rId10"/>
+    <sheet name="SatelliteLocation" sheetId="8" r:id="rId11"/>
+    <sheet name="LiveView" sheetId="9" r:id="rId12"/>
+    <sheet name="GeneratorInformation" sheetId="7" r:id="rId13"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1359" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="891">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -2581,47 +2577,155 @@
     <t>Email with valid format</t>
   </si>
   <si>
-    <t>Email with Alphabets</t>
-  </si>
-  <si>
-    <t>Email with Numbers</t>
-  </si>
-  <si>
-    <t>Email with Specialcharacters</t>
+    <t>henrry123@gmail.com</t>
+  </si>
+  <si>
+    <t>henrry123#@gmail,com</t>
+  </si>
+  <si>
+    <t>Henry123!@</t>
+  </si>
+  <si>
+    <t>Email with sepcialcharacters</t>
+  </si>
+  <si>
+    <t>Email with combination of char</t>
+  </si>
+  <si>
+    <t>hgf23#@</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email with Valid input </t>
+  </si>
+  <si>
+    <t>Email with Invalid input</t>
+  </si>
+  <si>
+    <t>Password with numbers</t>
+  </si>
+  <si>
+    <t>Password with specialcharacters</t>
+  </si>
+  <si>
+    <t>Password with combination of char</t>
+  </si>
+  <si>
+    <t>Password with Valid input</t>
+  </si>
+  <si>
+    <t>Forgot password with valid email</t>
+  </si>
+  <si>
+    <t>Forgot Password with Invalid email</t>
+  </si>
+  <si>
+    <t>First name with alphabets</t>
+  </si>
+  <si>
+    <t>First name with numbers</t>
+  </si>
+  <si>
+    <t>First name with specialcharacters</t>
+  </si>
+  <si>
+    <t>First name with combination of char</t>
+  </si>
+  <si>
+    <t>Joy@#231</t>
+  </si>
+  <si>
+    <t>First name with valid Input</t>
+  </si>
+  <si>
+    <t>Last name with alphabets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last name with numbers </t>
+  </si>
+  <si>
+    <t>Last name with specialcharacters</t>
+  </si>
+  <si>
+    <t>Last name with combination of char</t>
+  </si>
+  <si>
+    <t>Last name with valid input</t>
+  </si>
+  <si>
+    <t>Joy@#2123</t>
+  </si>
+  <si>
+    <t>Joy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone number with alphbets </t>
+  </si>
+  <si>
+    <t>Phone numbers with numbers</t>
+  </si>
+  <si>
+    <t>Phone numbers with specialcharacters</t>
+  </si>
+  <si>
+    <t>Phone number with more than 10 digits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone number with short input </t>
+  </si>
+  <si>
+    <t>987656787679</t>
+  </si>
+  <si>
+    <t>7890</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company name with alphbets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company name with numbers </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company name with specialcharacters </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zipcode with alphabets </t>
+  </si>
+  <si>
+    <t>zipcode with specialcharacters</t>
   </si>
   <si>
     <t>TC_007</t>
   </si>
   <si>
-    <t>765677</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Password with Alphabets </t>
-  </si>
-  <si>
-    <t>Password with Numbers</t>
-  </si>
-  <si>
-    <t>henrry123@gmail.com</t>
-  </si>
-  <si>
-    <t>henrry123#@gmail,com</t>
-  </si>
-  <si>
-    <t>Password with Specialcharacters</t>
-  </si>
-  <si>
-    <t>Password with all Characters</t>
-  </si>
-  <si>
-    <t>Henry123!@</t>
+    <t>TC_039</t>
+  </si>
+  <si>
+    <t>TC_050</t>
+  </si>
+  <si>
+    <t>TC_056</t>
+  </si>
+  <si>
+    <t>TC_67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account number with alphabets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account number with numbers </t>
+  </si>
+  <si>
+    <t>Account number with specialcharacters</t>
+  </si>
+  <si>
+    <t>9876543219</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2636,6 +2740,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF17C6A3"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2671,7 +2781,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -2707,6 +2817,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2723,10 +2834,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2991,71 +3098,809 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E87A73-4AF8-4170-BB53-1F60426C3268}">
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="40.28515625" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" customWidth="1"/>
+    <col min="6" max="6" width="40.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>136</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>4</v>
+        <v>137</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>6</v>
+        <v>846</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>8</v>
+        <v>847</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>9</v>
+        <v>849</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>882</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+        <v>320</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>256</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
+        <v>238</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>848</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
+        <v>843</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>743</v>
+      </c>
+      <c r="B5" t="s">
+        <v>320</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" t="s">
+        <v>845</v>
+      </c>
+      <c r="F5" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>883</v>
+      </c>
+      <c r="B8" t="s">
+        <v>843</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>884</v>
+      </c>
+      <c r="B11" t="s">
+        <v>320</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D11" t="s">
+        <v>238</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>861</v>
+      </c>
+      <c r="F11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>885</v>
+      </c>
+      <c r="B14" t="s">
+        <v>320</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D14" t="s">
+        <v>238</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>720</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>353</v>
+      </c>
+      <c r="B17" t="s">
+        <v>320</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D17" t="s">
+        <v>238</v>
+      </c>
+      <c r="E17" t="s">
+        <v>843</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>886</v>
+      </c>
+      <c r="B20" t="s">
+        <v>320</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>890</v>
+      </c>
+      <c r="D20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>875</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>280</v>
+      </c>
+      <c r="B23" t="s">
+        <v>320</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D23" t="s">
+        <v>238</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>880</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>286</v>
+      </c>
+      <c r="B26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D26" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>291</v>
+      </c>
+      <c r="B29" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D29" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C32" s="1"/>
+    </row>
+    <row r="34" spans="3:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C35" s="1"/>
+    </row>
+    <row r="37" spans="3:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C38" s="1"/>
+    </row>
+    <row r="40" spans="3:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C41" s="1"/>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="43" spans="3:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+    </row>
+    <row r="46" spans="3:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{463CF7D9-3797-4CC4-B6ED-F6CC315D9A0E}"/>
+    <hyperlink ref="C8" r:id="rId2" xr:uid="{364F7B74-6CD4-4433-B181-C5F191338975}"/>
+    <hyperlink ref="E11" r:id="rId3" xr:uid="{A96046E8-840F-4B16-A025-DD92433F934E}"/>
+    <hyperlink ref="E14" r:id="rId4" xr:uid="{7D47DDB9-53FA-4627-8621-375CB3198139}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77AFD7FA-CE31-4CAB-9D77-EB9A0F5923D7}">
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="65.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="6" width="40.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>322</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C5" t="s">
+        <v>320</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B8" t="s">
+        <v>333</v>
+      </c>
+      <c r="C8" t="s">
+        <v>320</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>255</v>
+      </c>
+      <c r="B11" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11" t="s">
+        <v>320</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E11" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>339</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C14" t="s">
+        <v>320</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E14" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>349</v>
+      </c>
+      <c r="B17" t="s">
+        <v>350</v>
+      </c>
+      <c r="C17" t="s">
+        <v>320</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E17" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>353</v>
+      </c>
+      <c r="B20" t="s">
+        <v>357</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>360</v>
+      </c>
+      <c r="B23" t="s">
+        <v>365</v>
+      </c>
+      <c r="C23" t="s">
+        <v>320</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E23" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>366</v>
+      </c>
+      <c r="B26" t="s">
+        <v>371</v>
+      </c>
+      <c r="C26" t="s">
+        <v>320</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E26" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>376</v>
+      </c>
+      <c r="B29" t="s">
+        <v>377</v>
+      </c>
+      <c r="C29" t="s">
+        <v>320</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E29" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>380</v>
+      </c>
+      <c r="B32" t="s">
+        <v>379</v>
+      </c>
+      <c r="C32" t="s">
+        <v>320</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E32" t="s">
+        <v>238</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B14" r:id="rId1" display="TRK@5678" xr:uid="{F0865D1B-BE06-4DAD-8D3E-B3E810C5D8FA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
   <dimension ref="A1:H106"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4569,7 +5414,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B8B5A6-41F7-4B76-9B90-A5C1587D6738}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4598,7 +5443,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
   <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5135,102 +5980,72 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0512D46C-65A2-499B-8C92-EB4BEF7A1CC2}">
-  <dimension ref="CY1:DD5"/>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="104" max="104" width="24.85546875" customWidth="1"/>
-    <col min="105" max="105" width="23.42578125" customWidth="1"/>
-    <col min="106" max="106" width="34.7109375" customWidth="1"/>
-    <col min="107" max="107" width="29.28515625" customWidth="1"/>
-    <col min="108" max="108" width="26" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="103:108" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="CY1" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="CZ1" s="3" t="s">
-        <v>843</v>
-      </c>
-      <c r="DA1" s="3" t="s">
-        <v>844</v>
-      </c>
-      <c r="DB1" s="3" t="s">
-        <v>845</v>
-      </c>
-      <c r="DC1" s="3" t="s">
-        <v>842</v>
-      </c>
-      <c r="DD1" s="3" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="2" spans="103:108" x14ac:dyDescent="0.25">
-      <c r="CY2" t="s">
-        <v>846</v>
-      </c>
-      <c r="CZ2" t="s">
-        <v>320</v>
-      </c>
-      <c r="DA2" s="1" t="s">
-        <v>847</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>238</v>
-      </c>
-      <c r="DC2" s="2" t="s">
-        <v>850</v>
-      </c>
-      <c r="DD2" s="2" t="s">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="4" spans="103:108" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="CY4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="CZ4" s="3" t="s">
-        <v>848</v>
-      </c>
-      <c r="DA4" s="3" t="s">
-        <v>849</v>
-      </c>
-      <c r="DB4" s="3" t="s">
-        <v>852</v>
-      </c>
-      <c r="DC4" s="3" t="s">
-        <v>853</v>
-      </c>
-    </row>
-    <row r="5" spans="103:108" x14ac:dyDescent="0.25">
-      <c r="CY5" t="s">
-        <v>743</v>
-      </c>
-      <c r="CZ5" t="s">
-        <v>320</v>
-      </c>
-      <c r="DA5" s="1" t="s">
-        <v>847</v>
-      </c>
-      <c r="DB5" t="s">
-        <v>238</v>
-      </c>
-      <c r="DC5" t="s">
-        <v>854</v>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="DD2" r:id="rId1" xr:uid="{94B42F2C-7046-4CDC-A622-B6682B8F51EB}"/>
-    <hyperlink ref="DC2" r:id="rId2" xr:uid="{F2801E8D-6087-460A-A710-A7B5F06DC167}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77142416-745D-4F9D-B8CB-E786E8AF6BF4}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5272,7 +6087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C6CDDE-28EE-4E4D-95AF-5786FC71BBC0}">
   <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5418,7 +6233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB07B270-85DC-4F6D-8AC7-D93CAE493508}">
   <dimension ref="A1:G42"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6035,7 +6850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16196D24-437F-4113-984C-E1E07E6FEFBB}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6088,7 +6903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A4B5976-09F6-46A1-AF3B-E9A8DFB4EAF3}">
   <dimension ref="A1:G68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6880,7 +7695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B476B142-4B93-4B5F-AFDD-C5C6F475C99C}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7032,7 +7847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58630B64-2EDF-4356-94B8-66DDB845E6F8}">
   <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7538,403 +8353,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77AFD7FA-CE31-4CAB-9D77-EB9A0F5923D7}">
-  <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="65.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" customWidth="1"/>
-    <col min="5" max="6" width="40.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>245</v>
-      </c>
-      <c r="B2" t="s">
-        <v>319</v>
-      </c>
-      <c r="C2" t="s">
-        <v>320</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>322</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="C5" t="s">
-        <v>320</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E5" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>328</v>
-      </c>
-      <c r="B8" t="s">
-        <v>333</v>
-      </c>
-      <c r="C8" t="s">
-        <v>320</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E8" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>255</v>
-      </c>
-      <c r="B11" t="s">
-        <v>338</v>
-      </c>
-      <c r="C11" t="s">
-        <v>320</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E11" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>339</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="C14" t="s">
-        <v>320</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E14" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>349</v>
-      </c>
-      <c r="B17" t="s">
-        <v>350</v>
-      </c>
-      <c r="C17" t="s">
-        <v>320</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E17" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>353</v>
-      </c>
-      <c r="B20" t="s">
-        <v>357</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="D20" t="s">
-        <v>238</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>360</v>
-      </c>
-      <c r="B23" t="s">
-        <v>365</v>
-      </c>
-      <c r="C23" t="s">
-        <v>320</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E23" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>366</v>
-      </c>
-      <c r="B26" t="s">
-        <v>371</v>
-      </c>
-      <c r="C26" t="s">
-        <v>320</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E26" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>374</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>376</v>
-      </c>
-      <c r="B29" t="s">
-        <v>377</v>
-      </c>
-      <c r="C29" t="s">
-        <v>320</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E29" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>380</v>
-      </c>
-      <c r="B32" t="s">
-        <v>379</v>
-      </c>
-      <c r="C32" t="s">
-        <v>320</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E32" t="s">
-        <v>238</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B14" r:id="rId1" display="TRK@5678" xr:uid="{F0865D1B-BE06-4DAD-8D3E-B3E810C5D8FA}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Modified test cases of generator portal login
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{0BC689DE-60D1-4641-9AF1-C6A0A8F0DCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{64C85B16-E0BF-4931-B17A-3CF7A51E25F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>